<commit_message>
[0814] 이더넷 reboot issue
</commit_message>
<xml_diff>
--- a/Protocol/Shelter_Protocol.xlsx
+++ b/Protocol/Shelter_Protocol.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로토콜 정의" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통신 흐름" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="동작 규칙" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="연결상태" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="동작 규칙" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설치·프로비저닝" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -145,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -183,6 +185,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -550,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -578,7 +583,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>rev 2.0</t>
+          <t>rev 2.5</t>
         </is>
       </c>
     </row>
@@ -590,7 +595,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
@@ -614,448 +619,370 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/state: ip 필드 제거 → uid (24hex) | LAN·브로커: 펌웨어 config.h</t>
+          <t>v2.5: DEV_RESET 소프트 리부트 · PB 릴레이 200ms · stat/pb conn 규칙 · CMS PB b_id 게이트</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>펌웨어 설정</t>
+          <t>PB b_id</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>control_board/code_mosquitto_choi/Core/Inc/config.h</t>
+          <t>전원보드 DIP 4bit → RS485 byte[1] → 제어보드 학습 → MQTT tele/stat (고정 1 아님)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>장치 식별</t>
+          <t>펌웨어 설정</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/state ONLINE 시 uid (STM32 96-bit UID)</t>
+          <t>config.h = Flash empty 시 fallback · 실제 설정은 직결 HTTP / Flash</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>LAN</t>
+          <t>장치 식별</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>config.h — STATIC {a,b,c,d} 또는 DHCP (MQTT에 IP 미포함)</t>
+          <t>dev/tele/state ONLINE 시 uid (STM32 96-bit UID)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>브로커 IP</t>
+          <t>LAN (현장)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>192.168.0.100 : 1883 (config.h SHELTER_MQTT_BROKER_IP)</t>
+          <t>Flash 저장 DHCP(권장) 또는 STATIC · 직결 HTTP로 최초 설정</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>참고 MD</t>
+          <t>브로커 IP</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Protocol/Shelter_Protocol.md (상세·미구현 항목)</t>
+          <t>직결 HTTP 또는 Flash · CMS 유지보수 / set_broker (원격)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>자동 보고</t>
+          <t>직결 프로비저닝</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>10분 주기 (재연결·명령 후 즉시 1회 + 타이머 리셋)</t>
+          <t>MQTT 90s 실패 → http://192.168.0.100 · PC=192.168.0.10 · HTML 내장</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>전원보드</t>
+          <t>설치 가이드</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>RS485 1초 보고 → MQTT 집계</t>
+          <t>Protocol/Shelter_Installation_Guide.md (설치 업체용)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>토픽 prefix</t>
+          <t>참고 MD</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/*  dev/stat/*  dev/cmnd/*</t>
+          <t>Protocol/Shelter_Protocol.md (MQTT 상세·미구현 항목)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>자동 보고</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>10분 주기 (재연결·명령 후 즉시 1회 + 타이머 리셋)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>전원보드</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>RS485 ~0.8s 폴링 → MQTT tele 10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>토픽 prefix</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>dev/tele/*  dev/stat/*  dev/cmnd/*</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>페이로드</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>JSON (UTF-8), QoS 0</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>■ 통신 방향 (토픽 구조)</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>방향</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Prefix</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>토픽 예시</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>발행 주체</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>구독 주체</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>장치 → 서버</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>dev/tele/</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>dev/tele/dust</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>제어보드</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>웹서버/브로커</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Telemetry · 10분 자동 보고</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>장치 → 서버</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>dev/stat/</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>dev/stat/pb</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>제어보드</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>웹서버/브로커</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>명령 처리 결과 (result 포함)</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>서버 → 장치</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>dev/cmnd/</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>dev/cmnd/pb</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>웹서버</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>제어보드</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>제어 명령 (dev/cmnd/# 구독)</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>■ 장치 목록 (7종 + 시스템)</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>장치</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>약어</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>tele</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>stat</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>cmnd</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>장비 상태</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>state</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>LWT OFFLINE</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>먼지센서</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>dust</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>tele 전용</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>내부 온습도</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>th_in</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>tele 전용</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>외부 온습도</t>
+          <t>장비 상태</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>th_out</t>
+          <t>state</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1075,7 +1002,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>tele 전용</t>
+          <t>LWT OFFLINE</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
@@ -1083,17 +1010,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>자동문 릴레이</t>
+          <t>먼지센서</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>dust</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1103,17 +1030,17 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>15채널</t>
+          <t>tele 전용</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr"/>
@@ -1121,17 +1048,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>내부 팬</t>
+          <t>내부 온습도</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>fan</t>
+          <t>th_in</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1141,17 +1068,17 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>AUTO/MANUAL</t>
+          <t>tele 전용</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -1159,17 +1086,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>전원보드</t>
+          <t>외부 온습도</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>pb</t>
+          <t>th_out</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1179,17 +1106,17 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>8채널 · MOS/TLS 공용</t>
+          <t>tele 전용</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -1197,17 +1124,17 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>공기청정기</t>
+          <t>자동문 릴레이</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ap</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1227,7 +1154,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Himpel</t>
+          <t>15채널</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
@@ -1235,17 +1162,17 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>에어컨(LG)</t>
+          <t>내부 팬</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>fan</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1265,7 +1192,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Modbus</t>
+          <t>AUTO/MANUAL · rpm · 타코 conn</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -1273,59 +1200,214 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>전원보드</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>pb</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>8채널 · MOS/TLS 공용</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>공기청정기</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>ap</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Himpel</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>에어컨(LG)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Modbus</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>시스템</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>dev</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>RESET / ALL_DATA</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>RESET / ALL_DATA / NET</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>외부 입력 4ch</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>PD4~PD7 · 보드 부착</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="19">
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B11:H11"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="B14:H14"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B17:H17"/>
     <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1337,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1779,12 +1861,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>{"mode":"MANUAL","duty":50,"conn":1}</t>
+          <t>{"mode":"MANUAL","duty":50,"rpm":1234,"conn":1}</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>{"fan":0,"conn":0}</t>
+          <t>{"fan":0,"rpm":0,"conn":0}</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -1807,12 +1889,15 @@
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>mode: AUTO|MANUAL
-duty: 0~100 [%]</t>
+duty: 0~100 [%]
+rpm: 타코 RPM</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>AUTO: 내부온도 기반</t>
+          <t>conn: duty≥10%→7s 타코
+duty&lt;10%→60s 이력
+AUTO: 내부온도</t>
         </is>
       </c>
     </row>
@@ -1831,12 +1916,12 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>{"mode":"MANUAL","duty":50,"conn":1,"result":1}</t>
+          <t>{"mode":"MANUAL","duty":50,"rpm":1234,"conn":1,"result":1}</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>{"fan":0,"conn":0,"result":1}</t>
+          <t>{"fan":0,"rpm":0,"conn":0,"result":1}</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -1886,7 +1971,7 @@
       <c r="D12" s="9" t="inlineStr">
         <is>
           <t>{
-  "b_id":1,
+  "b_id":3,
   "pb":[
     {"ch":1,"sw":1,"c":1.14,"w":250.8,"v":220},
     {"ch":2,"sw":1,"c":1.04,"w":228.5,"v":220},
@@ -1908,9 +1993,10 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>① {"b_id":1,"ch":1,"sw":1}
-② {"b_id":1,"set_pb":"11001101"}
-③ {"b_id":1,"get_pb":"state"}</t>
+          <t>① {"b_id":N,"ch":1,"sw":1}
+② {"b_id":N,"set_pb":"11001101"}
+③ {"b_id":N,"get_pb":"state"}
+(N=tele/get_pb 실측 b_id)</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -1920,15 +2006,18 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>b_id: 보드ID
+          <t>b_id: DIP 4bit(0~15)
+PB RS485 byte[1]
+제어보드 학습값
 ch:1~8 sw:0/1
 c[A] w[W] v[V]</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>RS485 1초 → conn 감지
-power_board 공용</t>
+          <t>RS485 ~0.8s 폴링
+MQTT tele 10s
+conn: HAL_OK / 10회 fail</t>
         </is>
       </c>
     </row>
@@ -1953,7 +2042,7 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>{"b_id":1,"pb":0,"conn":1,"result":0}</t>
+          <t>{"b_id":N,"pb":0,"conn":1,"result":0}</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
@@ -1982,7 +2071,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="150" customHeight="1">
+    <row r="14" ht="135" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>공기
@@ -2004,7 +2093,7 @@
         <is>
           <t>{"pwr":1,"mode":"AUTO","spd":3,"uv":1,
 "co2":450,"pm25":15,"pm10":20,"pm1_0":10,
-"temp":23.5,"humi":45,"filter":100,"conn":1}</t>
+"temp":23.5,"temp_out":18.2,"humi":45,"tvoc":120,"filter":100,"conn":1}</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2019,31 +2108,33 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>개별:
+          <t>개별·복합:
 {"pwr":0} {"mode":"AUTO"}
 {"spd":4} {"uv":1}
-{"filter_reset":1}
-{"bypass":1} {"timer":60}
+{"pwr":1,"mode":"AUTO","spd":2}
 일괄:
-{"set_ap":{"pwr":1,"mode":"AUTO","spd":4,"uv":1,"filter_reset":0,"bypass":0,"timer":0}}
+{"set_ap":{...}}
 조회:
 {"get_ap":"state"}</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>개별 7종 / set_ap / get_ap</t>
+          <t>개별·복합 / set_ap / get_ap</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>pwr 0/1, spd 1~4
-uv, co2, pm*, filter</t>
+          <t>pwr 0/1, spd 0~4
+mode: AUTO/MANUAL/CLEAN/VENT/BYPASS/HEATER
+temp, temp_out, tvoc</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Modbus Himpel</t>
+          <t>Himpel RS485
+(Modbus 아님)
+conn: RS485 OK</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2188,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="120" customHeight="1">
+    <row r="16" ht="135" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
           <t>에어컨
@@ -2131,29 +2222,32 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>개별:
+          <t>개별·복합:
 {"pwr":1} {"mode":"COOL"}
 {"temp":26} {"spd":3}
+{"pwr":1,"mode":"COOL","temp":24,"spd":2}
 일괄:
-{"set_ac":{"pwr":1,"mode":"COOL","temp":26,"spd":3}}
+{"set_ac":{...}}
 조회:
 {"get_ac":"state"}</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>개별 4종 / set_ac / get_ac</t>
+          <t>개별·복합 / set_ac / get_ac</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>mode: COOL/HEAT/FAN/DRY
-temp 16~30, err:0=정상</t>
+          <t>mode: COOL/HEAT/FAN/DRY/AUTO
+temp 16~30, spd 1~6</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Modbus RTU LG</t>
+          <t>LG Modbus RTU
+conn: Discrete
+ADDR_AC_CONN bit</t>
         </is>
       </c>
     </row>
@@ -2207,70 +2301,191 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="75" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>외부
+입력
+(4ch)</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>tele</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>dev/tele/input</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>{"in":[1,0,0,1],"count":[12,0,0,3],"conn":1}</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>(보드 부착 —
+미연결 없음)</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>dev/cmnd/input</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>① {"get_input":"state"}
+② {"reset_count":1}</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>조회 / 카운트 초기화</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>in: PD4~PD7 [0/1]
+count: 상승엣지 누적
+conn: 1 (보드 부착)</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>상태변경 즉시 dev/tele/input
+(서버 폴링 없음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>stat
+(응답)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>dev/stat/input</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>{"in":[1,0,0,1],"count":[12,0,0,3],"conn":1,"result":1}</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>{"in":[0,0,0,0],"count":[0,0,0,0],"conn":1,"result":0}</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>dev/cmnd/input</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>(위 cmnd 참조)</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>get_input / reset_count 응답</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>result: 1/0</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>연결 표시 불필요 (보드 GPIO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="345" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>시스템
 제어</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>stat
 (응답)</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>dev/stat/dev</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>{"device":"ALL_DATA","conn":1,"result":1}
 + tele 8종 일괄 발행</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>{"device":"DEV_RESET","conn":0,"result":1}</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>dev/cmnd/dev</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>① {"reset":"DEV_RESET"}
-   → 500ms 후 리부팅
+   → 500ms 후 소프트 리부트
+     (Flash·네트워크 유지)
 ② {"data":"ALL_DATA"}
    → stat ACK +
-     tele 전체 즉시 발행</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>리셋 / 전체 데이터</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
+     tele 전체 즉시 발행
+③ {"set_net":{"ip":[...],"sn":[...],"gw":[...]}}
+   → STATIC IP Flash 저장
+④ {"set_broker":{"ip":[...],"port":1883}}
+   → 브로커 Flash 저장
+⑤ {"set_net_reset":1}
+   → Flash DHCP 공장 초기화
+⑥ 직결 HTTP (v2.1)
+   → 192.168.0.100:80
+     PC 192.168.0.10
+⑦ {"clear_net":1} (예정)
+⑧ {"clear_broker":1} (예정)</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>리셋 / 전체 / NET / 브로커</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>ALL_DATA 발행:
 th_in, th_out, dust,
-ad, fan, ac, pb, ap</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>서버 최초 연결 시
-ALL_DATA 권장</t>
+ad, fan, ac, pb, ap, input</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>clear_* : 자체 8ch 스위치
+별도 제어보드 IP/브로커
+삭제 (펌웨어 예정)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A12:A13"/>
@@ -2280,6 +2495,7 @@
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="A14:A15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2292,7 +2508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2470,322 +2686,330 @@
       </c>
       <c r="F8" s="3" t="inlineStr"/>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>외부 입력 4ch</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>장치→서버</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>dev/tele/input</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>{"in":[1,0,0,1],"count":[12,0,0,3],"conn":1}</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>상태변경 즉시</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>PD4~PD7 · 연결 표시 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>■ B. 제어 장비 — 양방향 (cmnd → stat, tele 자동 보고)</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>장치</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>서버→장치 (cmnd)</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>장치→서버 (stat)</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>장치→서버 (tele)</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>흐름</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>AD (릴레이 15ch)</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>dev/cmnd/ad</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>dev/stat/ad</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>dev/tele/ad</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>서버 ──cmnd──▶ 장치 ──stat──▶ 서버
 장치 ──tele──▶ 서버 (10분)</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>15채널 릴레이</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Fan (팬)</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>dev/cmnd/fan</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>dev/stat/fan</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>dev/tele/fan</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>set_fan / get_fan</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>AUTO/MANUAL duty 0~100</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>PB (전원 8ch)</t>
+          <t>Fan (팬)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>dev/cmnd/pb</t>
+          <t>dev/cmnd/fan</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>dev/stat/pb</t>
+          <t>dev/stat/fan</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/pb</t>
+          <t>dev/tele/fan</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>set_pb(8자리) / get_pb</t>
+          <t>set_fan / get_fan</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>RS485 1초 · MOS/TLS 공용</t>
+          <t>AUTO/MANUAL · rpm · 타코 conn</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>AP (공기청정)</t>
+          <t>PB (전원 8ch)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>dev/cmnd/ap</t>
+          <t>dev/cmnd/pb</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>dev/stat/ap</t>
+          <t>dev/stat/pb</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/ap</t>
+          <t>dev/tele/pb</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>set_ap / 개별 pwr,mode,spd…</t>
+          <t>set_pb(8자리) / get_pb</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Himpel Modbus</t>
+          <t>RS485 ~0.8s · tele 10s</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>AC (에어컨)</t>
+          <t>AP (공기청정)</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>dev/cmnd/ac</t>
+          <t>dev/cmnd/ap</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>dev/stat/ac</t>
+          <t>dev/stat/ap</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/ac</t>
+          <t>dev/tele/ap</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>set_ac / 개별 pwr,mode,temp…</t>
+          <t>set_ap / 개별·복합 pwr,mode,spd…</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>LG Modbus RTU</t>
+          <t>Himpel RS485</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>AC (에어컨)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>dev/cmnd/ac</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>dev/stat/ac</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>dev/tele/ac</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>set_ac / 개별 pwr,mode,temp…</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>LG Modbus RTU</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>DEV (시스템)</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>dev/cmnd/dev</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>dev/stat/dev</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>(없음)</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>RESET / ALL_DATA → tele 8종 일괄</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>서버 최초 연결 시 ALL_DATA</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>■ C. ALL_DATA 시퀀스</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>순서</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>방향</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>토픽</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Payload / 동작</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>서버→장치</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>dev/cmnd/dev</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>{"data":"ALL_DATA"}</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>장치→서버</t>
+          <t>서버→장치</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>dev/stat/dev</t>
+          <t>dev/cmnd/dev</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>{"device":"ALL_DATA","conn":1,"result":1}</t>
+          <t>{"data":"ALL_DATA"}</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr"/>
@@ -2794,7 +3018,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2804,12 +3028,12 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>dev/tele/th_in ~ ap</t>
+          <t>dev/stat/dev</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>각 tele 토픽 즉시 1회 발행 (8종)</t>
+          <t>{"device":"ALL_DATA","conn":1,"result":1}</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
@@ -2818,33 +3042,57 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>장치→서버</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>dev/tele/th_in ~ ap</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>10분 타이머 전체 리셋</t>
+          <t>각 tele 토픽 즉시 1회 발행 (8종)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>10분 타이머 전체 리셋</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2856,7 +3104,559 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>conn — 연결됨 / 오프라인 판정 (rev 2.2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>CMS UI 배지 = 각 tele/stat의 conn 필드. 메인보드 MQTT 수신 시 하위 장치 conn 을 일괄 1로 만들지 않음.</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>장치</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>conn=1 (펌웨어)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>conn=0 / 미연결 payload</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>CMS 표시</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>타임아웃·주기</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>state
+(메인보드)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>MQTT 브로커 연결</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>{"status":"OFFLINE"} (LWT)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>state.conn=1 (MQTT 수신)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>5분 무수신→OFFLINE</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>uid/ip/mode 포함</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>dust</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>UART 패킷 수신·60s 이내 갱신</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>{"dust":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>tele 10분</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>UPDM010UB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>th_in</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>HC-SD Modbus OK + 유효 온도</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>{"thindoor":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>읽기 3s · fail×30</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>내부 온습</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>th_out</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>CWT-TH03S Modbus OK</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>{"thoutdoor":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>읽기 2.5s · fail×10</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>외부 온습</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>제어보드 릴레이 (항상 부착)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn=1</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>tele 10분</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>미연결 개념 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>fan</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>duty≥10%: 타코 7s 이내
+ duty&lt;10%: 60s 이력</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>{"fan":0,"rpm":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn + rpm</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>conn 변경 즉시</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>TIM1 CH3 타코</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>pb</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>RS485 UpdateAllData HAL_OK</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>{"b_id":N,"pb":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>pb[]+conn; graph 35s stale</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>tele 10s · fail×10</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>전원보드 RS485</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ap</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Himpel RS485 응답 OK</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>{"ap":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>10s 무응답→0</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>공기청정기</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Modbus Discrete ADDR_AC_CONN
+읽기 OK 且 bit=1</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>{"ac":0,"conn":0}</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>payload.conn</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>폴링 ~1s</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>LG Modbus</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>PD4~PD7 GPIO</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>(없음)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>conn=1</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>변경 즉시</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>외부 입력 4ch</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>■ CMS (server.js) 요약</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>기능</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>동작</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>normalizeConn</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>tele/stat JSON conn 필드만 0/1 변환</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>기본값 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>resetDeviceTimeout</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>아무 MQTT 수신 → state.conn=1, 5분 타이머</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>하위 conn 일괄 변경 X</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>setAllOffline</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>5분 무수신 → state OFFLINE, dust/th/ad/fan/ap/ac/input conn=0</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>pb 키 제외</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>PB tele</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>pb[] 배열 + conn → conn=1; pb:0 → conn=0 (tele에 result 없음)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>PB_TELE_STALE_MS=35s</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>PB b_id</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>current_b_id 초기 0 — tele 수신 후 캐시</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>하드코딩 금지</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>스케줄</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>출근 set_ac / set_ap 일괄 명령</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>stat result:0</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>해당 장치 conn=0</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>명령 실패 반영</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2929,12 +3729,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>tele 토픽 순차 발행. PB는 RS485 1초 + MQTT</t>
+          <t>tele 순차. PB: RS485 ~0.8s + MQTT 10s</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>전원보드 conn 감지</t>
+          <t>전원보드 conn</t>
         </is>
       </c>
     </row>
@@ -3039,6 +3839,182 @@
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>직결 프로비저닝</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>링크UP+IP없음 5s → 192.168.0.100 · 저장직후 pending=1 → LAN 2분</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>양산·최초설치 표준</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>설정 우선순위</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Flash &gt; config.h fallback</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>CMS=유지보수</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>conn 독립 (v2.2)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>장치별 tele conn만 UI. 메인 MQTT ≠ 전체 연결</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>CMS server.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>CMS 메인 타임아웃</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>5분 MQTT 없음 → state OFFLINE + 하위 conn=0</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>DEVICE_TIMEOUT_MS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>장치 conn 판정</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>dust 60s / fan 타코 / PB RS485×10 / AC discrete</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>시트 '연결상태'</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>복합 cmnd (v2.4)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>AC/AP JSON 다필드 순차 적용 · set_ac/set_ap 권장</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>mqtt_handler.c</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>tele vs stat</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>result는 stat 전용 · tele/pb에 result 없음</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>app.c</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>PB b_id</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>서버 b_id 하드코딩 금지 · 초기 0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>server.js</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3046,4 +4022,567 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Smart Shelter 설치·프로비저닝 (v2.1 — 설치 업체·양산)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>상세 절차: Protocol/Shelter_Installation_Guide.md</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>단계</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>작업</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>값 / URL</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>펌웨어</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>공통 이미지 플래시</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>code_mosquitto_choi</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>고객별 config.h 빌드 불필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>직결</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>PC ↔ 제어보드 이더넷</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>케이블 1m+</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>공유기 불필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>대기</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>설정 모드 진입</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>링크 UP + 5s</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>재설정·공장 / 케이블 필수</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>PC IP</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Windows 수동 IP</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>192.168.0.10 / 255.255.255.0</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Wi-Fi 끄기 권장</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>브라우저</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>설정 페이지</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>http://192.168.0.100</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>포트 80 · XML 불필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>LAN</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>모드 선택</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>DHCP (권장)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>STATIC = 고정 IP만</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>브로커</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>MQTT 입력</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>관제 PC LAN IP : 1883</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Flash 저장</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>저장</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>저장 및 재부팅</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>save.cgi → pending=1</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Flash → reboot</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>★ PC 케이블 분리 → LAN</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>공유기/스위치</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>2분 DHCP 유예</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>확인</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>CMS ONLINE</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>dev/tele/state uid</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>설치 완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>■ IP 요약</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>서브넷</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>제어보드 (직결)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>192.168.0.100</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>255.255.255.0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>프로비저닝 전용</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>설정 PC</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>192.168.0.10</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>255.255.255.0</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>수동 설정</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>제어보드 (현장)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>DHCP 할당</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>예: 192.168.0.x</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>공유기 LAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>MQTT 브로커</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>서버 LAN IP</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>포트 1883</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>MOS 비암호화</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>■ 공장 초기화 / 유지보수</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>방법</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>명령/동작</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>SW8</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Flash erase → DHCP 공장값</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>최초 설정 재진행</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>set_net_reset</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>{"set_net_reset":1}</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>MQTT — ONLINE 시</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>CMS 유지보수</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>🔧 네트워크 메뉴</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>최초 설치 X · 원격 변경용</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>